<commit_message>
Working code for Bridge and LBracketComplianceMassCost
</commit_message>
<xml_diff>
--- a/data/LBracketMaterialsSI.xlsx
+++ b/data/LBracketMaterialsSI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Personal\suresh\Software\Github\ERSL-Private\METALS\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73C75285-1D23-45C7-9080-1B617790709C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BF2CA57-1A1A-46BD-AD61-313FF533FC1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1920" yWindow="1776" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="23">
   <si>
     <t>Attribute</t>
   </si>
@@ -82,31 +82,25 @@
     <t>Grade 304 SS</t>
   </si>
   <si>
-    <t>Nitronic 60</t>
+    <t>6061 Al</t>
+  </si>
+  <si>
+    <t>USD/lb</t>
+  </si>
+  <si>
+    <t>USD/g</t>
+  </si>
+  <si>
+    <t>USD/kg</t>
+  </si>
+  <si>
+    <t>Attributes</t>
+  </si>
+  <si>
+    <t>Material/Units</t>
   </si>
   <si>
     <t>7068 Al</t>
-  </si>
-  <si>
-    <t>7075 Al</t>
-  </si>
-  <si>
-    <t>6061 Al</t>
-  </si>
-  <si>
-    <t>USD/lb</t>
-  </si>
-  <si>
-    <t>USD/g</t>
-  </si>
-  <si>
-    <t>USD/kg</t>
-  </si>
-  <si>
-    <t>Attributes</t>
-  </si>
-  <si>
-    <t>Material/Units</t>
   </si>
 </sst>
 </file>
@@ -476,7 +470,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.6640625" style="1" customWidth="1"/>
@@ -486,7 +480,7 @@
   <sheetData>
     <row r="1" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>4</v>
@@ -503,7 +497,7 @@
     </row>
     <row r="2" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>7</v>
@@ -512,7 +506,7 @@
         <v>12</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>12</v>
@@ -529,10 +523,10 @@
         <v>196000000000</v>
       </c>
       <c r="D3" s="2">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E3" s="5">
-        <v>1000000000</v>
+        <v>900000000</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -540,83 +534,49 @@
         <v>15</v>
       </c>
       <c r="B4" s="5">
-        <v>8000</v>
+        <v>7700</v>
       </c>
       <c r="C4" s="5">
         <v>193000000000</v>
       </c>
       <c r="D4" s="2">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="E4" s="5">
-        <v>230000000</v>
+        <v>700000000</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="5">
-        <v>7620</v>
-      </c>
-      <c r="C5" s="5">
-        <v>181000000000</v>
-      </c>
-      <c r="D5" s="2">
-        <v>4</v>
-      </c>
-      <c r="E5" s="5">
-        <v>689000000</v>
+      <c r="A5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="6">
+        <v>2850</v>
+      </c>
+      <c r="C5" s="6">
+        <v>73000000000</v>
+      </c>
+      <c r="D5" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="E5" s="6">
+        <v>590000000</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B6" s="6">
-        <v>2850</v>
+        <v>2700</v>
       </c>
       <c r="C6" s="6">
-        <v>73000000000</v>
+        <v>69000000000</v>
       </c>
       <c r="D6" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" s="6">
-        <v>590000000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="6">
-        <v>2810</v>
-      </c>
-      <c r="C7" s="6">
-        <v>72000000000</v>
-      </c>
-      <c r="D7" s="3">
-        <v>2</v>
-      </c>
-      <c r="E7" s="6">
-        <v>503000000</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" s="6">
-        <v>2700</v>
-      </c>
-      <c r="C8" s="6">
-        <v>69000000000</v>
-      </c>
-      <c r="D8" s="3">
-        <v>2</v>
-      </c>
-      <c r="E8" s="6">
         <v>276000000</v>
       </c>
     </row>
@@ -697,13 +657,13 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D4" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>